<commit_message>
Stage 8 fixes: G-012
</commit_message>
<xml_diff>
--- a/output/heldback_firm_G/OsterquillData/Studies/OT-26-S0177/Raw_Observations/Interim/BP16_Genotox_091826_INTERIM.xlsx
+++ b/output/heldback_firm_G/OsterquillData/Studies/OT-26-S0177/Raw_Observations/Interim/BP16_Genotox_091826_INTERIM.xlsx
@@ -567,7 +567,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>negative</t>
+          <t>negative for the completed bacterial phase; article identity and per-article record linkage [TBC]. Not a cohort-wide negative conclusion.</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>HepG2 cytotoxicity exclusion applied to the scoring of one mammalian condition. Repeat scoring XX% complete.</t>
+          <t>TK6 cytotoxicity/RPD assessment excluded a mammalian scoring condition. Article [TBC]; concentration [TBC]; treatment [TBC]; TK6 exclusion record under OQ/2026/002835 [TBC]. HepG2 ATP results are a separate preliminary screen and do not establish TK6 cytotoxicity. Repeat scoring XX% complete.</t>
         </is>
       </c>
     </row>
@@ -962,7 +962,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Control validity met for every strain on the day of scoring.</t>
+          <t>Bacterial phase complete. Rows are strain/dose conditions, not separate test articles. Negative outcome applies to the tested article in the bacterial phase report under OQ/2026/002835; article identity and linked per-article records [TBC]. Control validity met for the scored strains.</t>
         </is>
       </c>
     </row>
@@ -1878,7 +1878,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1988,6 +1988,19 @@
       </c>
       <c r="D6" s="2" t="inlineStr"/>
     </row>
+    <row r="7"/>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Exclusion source</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>TK6 cytotoxicity/RPD assessment under OQ/2026/002835; article [TBC], concentration [TBC], treatment [TBC], source-record reference [TBC]. HepG2 does not determine this exclusion.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>